<commit_message>
Added all queries for C3DC testcases
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC02_C3DC_phs000471_Race-Unknown.xlsx
+++ b/InputFiles/C3DC/TC02_C3DC_phs000471_Race-Unknown.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="35840" yWindow="-2240" windowWidth="30240" windowHeight="24500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -502,59 +502,39 @@
     <row r="2" ht="297" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>StudiesTab</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT
-     std.dbgap_accession AS "dbGaP Accession",
-     std.study_name AS "Study Name"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE 
-    std.dbgap_accession = 'phs000471' AND prt.race = 'Unknown'</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>SELECT 
-    COUNT(DISTINCT dgn.diagnosis) AS Diagnoses,
-    COUNT(DISTINCT prt.participant_id) AS Participants,
-    COUNT(DISTINCT std.study_id) AS Studies
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE 
-   std.dbgap_accession = 'phs000471' AND prt.race = 'Unknown';</t>
+          <t>ParticipantsTab</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000471'
+  AND 'Unknown' IN coalesce(p.race, [])
+RETURN p.participant_id AS `Participant ID`,
+       s.study_id AS `Study ID`,
+       p.sex_at_birth AS `Sex at Birth`,
+       reduce(text = '', value IN coalesce(p.race, []) | CASE WHEN text = '' THEN value ELSE text + '; ' + value END) AS `Race`
+ORDER BY p.participant_id
+LIMIT 100;</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000471'
+  AND 'Unknown' IN coalesce(p.race, [])
+OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(p)
+OPTIONAL MATCH (f)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file|of_radiology_file]-&gt;(sm)
+OPTIONAL MATCH (fp)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(p)
+RETURN count(DISTINCT s) AS studies,
+       count(DISTINCT p) AS participants,
+       count(DISTINCT sm) AS samples,
+       count(DISTINCT f) + count(DISTINCT fp) AS files</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TC02_C3DC_phs000471_Race-Unknown_TSVData.xlsx</t>
+          <t>TC02_C3DC_phs000471_Race-Unknown_DbData.xlsx</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -566,34 +546,86 @@
     <row r="3" ht="372" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ParticipantsTab</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT
-    prt.participant_id AS "Participant Id",
-    REPLACE(prt.race, ';', ', ') AS "Race",
-    prt.sex_at_birth AS "Sex at Birth",
-    std.dbgap_accession AS "dbGaP Accession"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE 
-    std.dbgap_accession = 'phs000471' AND prt.race = 'Unknown'
-ORDER BY 
-    prt.participant_id ASC
+          <t>StudiesTab</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MATCH (s:study)
+WHERE EXISTS {
+  MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+  WHERE s.dbgap_accession = 'phs000471' AND 'Unknown' IN coalesce(p.race, [])
+}
+WITH s
+MATCH (sp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, count(DISTINCT sp) AS num_of_participants
+OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, count(DISTINCT sm) AS num_of_samples
+OPTIONAL MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(dp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, d.diagnosis AS diagnosis_name, count(DISTINCT dp) AS diagnosis_n
+ORDER BY diagnosis_n DESC, diagnosis_name
+WITH s, num_of_participants, num_of_samples,
+     [item IN collect(CASE WHEN diagnosis_name IS NULL THEN null ELSE diagnosis_name + ' (' + toString(diagnosis_n) + ')' END) WHERE item IS NOT NULL] AS diagnosis_all
+WITH s, num_of_participants, num_of_samples,
+     diagnosis_all[0..5] AS diagnosis_items,
+     size(diagnosis_all) &gt; 5 AS diagnosis_more
+OPTIONAL MATCH (d2:diagnosis)-[:of_diagnosis]-&gt;(dp2:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+UNWIND CASE WHEN d2 IS NULL THEN [null] ELSE coalesce(d2.anatomic_site, [null]) END AS site
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(DISTINCT dp2) AS site_n
+ORDER BY site_n DESC, site
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
+     [item IN collect(CASE WHEN site IS NULL THEN null ELSE site + ' (' + toString(site_n) + ')' END) WHERE item IS NOT NULL] AS site_all
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
+     site_all[0..5] AS site_items,
+     size(site_all) &gt; 5 AS site_more
+OPTIONAL MATCH (sf)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file]-&gt;(:sample)-[:of_sample]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     sf.file_type AS file_type, count(DISTINCT sf) AS type_n
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     [item IN collect(CASE WHEN file_type IS NULL OR type_n = 0 THEN null ELSE {t: file_type, n: type_n} END) WHERE item IS NOT NULL] AS sample_file_types
+OPTIONAL MATCH (pf)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, sample_file_types,
+     pf.file_type AS file_type, count(DISTINCT pf) AS type_n
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, sample_file_types,
+     [item IN collect(CASE WHEN file_type IS NULL OR type_n = 0 THEN null ELSE {t: file_type, n: type_n} END) WHERE item IS NOT NULL] AS participant_file_types
+OPTIONAL MATCH (stf)-[:of_clinical_measure_file|of_generic_file]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, sample_file_types, participant_file_types,
+     stf.file_type AS file_type, count(DISTINCT stf) AS type_n
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     sample_file_types + participant_file_types + [item IN collect(CASE WHEN file_type IS NULL OR type_n = 0 THEN null ELSE {t: file_type, n: type_n} END) WHERE item IS NOT NULL] AS file_types
+UNWIND CASE WHEN size(file_types) = 0 THEN [{t: null, n: 0}] ELSE file_types END AS ft
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     ft.t AS file_type, sum(ft.n) AS type_n
+ORDER BY type_n DESC, file_type
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     sum(CASE WHEN file_type IS NULL THEN 0 ELSE type_n END) AS num_of_files,
+     [item IN collect(CASE WHEN file_type IS NULL THEN null ELSE file_type + ' (' + toString(type_n) + ')' END) WHERE item IS NOT NULL] AS file_type_all
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files,
+     file_type_all[0..5] AS file_type_items,
+     size(file_type_all) &gt; 5 AS file_type_more
+OPTIONAL MATCH (pub:publication)-[:of_publication]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files, file_type_items, file_type_more,
+     [id IN collect(pub.pubmed_id) WHERE id IS NOT NULL] AS pubmed_ids
+OPTIONAL MATCH (per:study_personnel)-[:of_study_personnel]-&gt;(s)
+WHERE per IS NULL OR per.personnel_type = 'PI'
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files, file_type_items, file_type_more, pubmed_ids,
+     [name IN collect(per.personnel_name) WHERE name IS NOT NULL] AS investigators
+OPTIONAL MATCH (fund:study_funding)-[:of_study_funding]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files, file_type_items, file_type_more, pubmed_ids, investigators,
+     [id IN collect(fund.grant_id) WHERE id IS NOT NULL] AS grant_ids
+RETURN s.study_name AS `Study Name`,
+       s.study_id AS `Study ID`,
+       s.study_phase AS `Study Phase`,
+       reduce(text = '', item IN diagnosis_items | CASE WHEN text = '' THEN item ELSE text + '\u000a' + item END) + CASE WHEN diagnosis_more THEN '\u000a' + 'Read More' ELSE '' END AS `Diagnosis (Top 5)`,
+       reduce(text = '', item IN site_items | CASE WHEN text = '' THEN item ELSE text + '\u000a' + item END) + CASE WHEN site_more THEN '\u000a' + 'Read More' ELSE '' END AS `Diagnosis Anatomic Site (Top 5)`,
+       toString(num_of_participants) AS `Number of Participants`,
+       toString(num_of_samples) AS `Number of Samples`,
+       toString(num_of_files) AS `Number of Files`,
+       reduce(text = '', item IN file_type_items | CASE WHEN text = '' THEN item ELSE text + '\u000a' + item END) + CASE WHEN file_type_more THEN '\u000a' + 'Read More' ELSE '' END AS `File Type (Top 5)`,
+       reduce(text = '', item IN pubmed_ids | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS `PubMed ID`,
+       reduce(text = '', item IN investigators | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS `Principal Investigator(s)`,
+       reduce(text = '', item IN grant_ids | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS `Grant ID`
+ORDER BY s.study_name
 LIMIT 100;</t>
         </is>
       </c>
@@ -604,225 +636,195 @@
           <t>DiagnosisTab</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT
-    prt.participant_id AS "Participant Id",
-    dgn.diagnosis_id AS "Diagnosis Id",
-    dgn.diagnosis AS "Diagnosis",
-    CASE 
-    WHEN dgn.age_at_diagnosis = -999 THEN 'Not Reported'
-    WHEN dgn.age_at_diagnosis &gt;= 1000 THEN 
-        substr(dgn.age_at_diagnosis, 1, length(dgn.age_at_diagnosis) - 3) || ',' || substr(dgn.age_at_diagnosis, -3)
-    ELSE 
-        dgn.age_at_diagnosis 
-END AS "Age at Diagnosis (days)",
-    dgn.anatomic_site AS "Anatomic Site",
-    dgn.diagnosis_classification_system AS "Diagnosis Classification System",
-    std.dbgap_accession AS "dbGaP Accession"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE 
-    std.dbgap_accession = 'phs000466' AND prt.sex_at_birth = 'Male' AND dgn.diagnosis_id IS NOT NULL
-ORDER BY 
-    prt.participant_id ASC
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000471'
+  AND 'Unknown' IN coalesce(p.race, [])
+RETURN p.participant_id AS `Participant ID`,
+       d.diagnosis_id AS `Diagnosis ID`,
+       d.diagnosis AS `Diagnosis`,
+       CASE
+         WHEN d.age_at_diagnosis IS NULL OR d.age_at_diagnosis = -999 THEN 'Not Reported'
+         ELSE toString(d.age_at_diagnosis)
+       END AS `Age at Diagnosis (days)`,
+       reduce(text = '', value IN coalesce(d.anatomic_site, []) | CASE WHEN text = '' THEN value ELSE text + ', ' + value END) AS `Anatomic Site`,
+       reduce(text = '', value IN coalesce(d.diagnosis_classification_system, []) | CASE WHEN text = '' THEN value ELSE text + ', ' + value END) AS `Diagnosis Classification System`,
+       s.dbgap_accession AS `dbGaP Accession`
+ORDER BY p.participant_id
 LIMIT 100;</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
     </row>
     <row r="5" ht="409.6" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TreatmentTab</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT
-    prt.participant_id AS "Participant Id",
-    trt.treatment_id AS "Treatment Id",
-    CASE 
-    WHEN trt.age_at_treatment_start = -999 THEN 'Not Reported'
-    WHEN trt.age_at_treatment_start &gt;= 1000 THEN 
-        substr(trt.age_at_treatment_start, 1, length(trt.age_at_treatment_start) - 3) || ',' || substr(trt.age_at_treatment_start, -3)
-    ELSE 
-        trt.age_at_treatment_start 
-END AS "Age at Treatment Start",
-    CASE 
-    WHEN trt.age_at_treatment_end = -999 THEN 'Not Reported'
-    WHEN trt.age_at_treatment_end &gt;= 1000 THEN 
-        substr(trt.age_at_treatment_end, 1, length(trt.age_at_treatment_end) - 3) || ',' || substr(trt.age_at_treatment_end, -3)
-    ELSE 
-        trt.age_at_treatment_end 
-END AS "Age at Treatment End",
-    trt.treatment_type AS "Treatment Type",
-    REPLACE(trt.treatment_agent, ';', ', ') AS "Treatment Agent",
-    std.dbgap_accession AS "dbGaP Accession"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE 
-    std.dbgap_accession = 'phs000471' AND prt.race = 'Unknown'
-ORDER BY 
-    trt.treatment_id ASC
+          <t>GeneticAnalysisTab</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MATCH (g:genetic_analysis)-[:of_genetic_analysis]-&gt;(:sample)-[:of_sample]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000471'
+  AND 'Unknown' IN coalesce(p.race, [])
+WITH p, g, s,
+     CASE
+       WHEN g.gene_symbol IS NULL THEN []
+       WHEN valueType(g.gene_symbol) = 'LIST' THEN g.gene_symbol
+       WHEN g.gene_symbol STARTS WITH '[' AND g.gene_symbol ENDS WITH ']'
+         THEN split(substring(g.gene_symbol, 1, size(g.gene_symbol) - 2), ', ')
+       ELSE [g.gene_symbol]
+     END AS genes
+RETURN p.participant_id AS `Participant ID`,
+       g.genetic_analysis_id AS `Genetic Analysis ID`,
+       reduce(text = '', item IN genes[0..5] | CASE WHEN text = '' THEN item ELSE text + '\u000a' + item END)
+         + CASE WHEN size(genes) &gt; 5 THEN '\u000a' + 'Read More' ELSE '' END AS `Gene Symbol (Top 5)`,
+       g.status AS `Status`,
+       g.reported_significance AS `Reported Significance`,
+       g.reported_significance_system AS `Reported Significance System`,
+       g.hgvs_genome AS `HGVS Genome`,
+       g.alteration AS `Alteration`,
+       s.study_id AS `Study ID`
+ORDER BY p.participant_id, g.genetic_analysis_id
 LIMIT 100;</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
     </row>
     <row r="6" ht="409.6" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TreatmentRespTab</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT
-    prt.participant_id AS "Participant Id",
-    trr.treatment_response_id AS "Treatment Response Id",
-    trr.response AS "Response",
-    CASE 
-        WHEN trr.age_at_response = -999 THEN 'Not Reported'
-        WHEN trr.age_at_response &gt;= 1000 THEN 
-            substr(trr.age_at_response, 1, length(trr.age_at_response) - 3) || ',' || substr(trr.age_at_response, -3)
-        ELSE 
-            trr.age_at_response 
-    END AS "Age at Response",
-    std.dbgap_accession AS "dbGaP Accession"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1   -- participants not directly linked to studies
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE
-    std.dbgap_accession = 'phs000466' AND prt.sex_at_birth = 'Male' and trr.treatment_response_id is not NULL
-ORDER BY 
-    prt.participant_id ASC
+          <t>TreatmentTab</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CALL {
+  MATCH (t:treatment_chemotherapy)-[:of_treatment_chemotherapy]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+  WHERE s.dbgap_accession = 'phs000471' AND 'Unknown' IN coalesce(p.race, [])
+  RETURN p.participant_id AS participant_id,
+         t.guid AS treatment_id,
+         CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
+         CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
+         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
+         reduce(text = '', item IN coalesce(t.chemotherapy_agent, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_agent,
+         s.dbgap_accession AS dbgap_accession
+  UNION
+  MATCH (t:treatment_radiation)-[:of_treatment_radiation]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+  WHERE s.dbgap_accession = 'phs000471' AND 'Unknown' IN coalesce(p.race, [])
+  RETURN p.participant_id AS participant_id,
+         t.guid AS treatment_id,
+         CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
+         CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
+         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
+         reduce(text = '', item IN coalesce(t.radiation_therapy_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_agent,
+         s.dbgap_accession AS dbgap_accession
+  UNION
+  MATCH (t:treatment_surgery)-[:of_treatment_surgery]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+  WHERE s.dbgap_accession = 'phs000471' AND 'Unknown' IN coalesce(p.race, [])
+  RETURN p.participant_id AS participant_id,
+         t.guid AS treatment_id,
+         CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
+         CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
+         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
+         reduce(text = '', item IN coalesce(t.surgery_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_agent,
+         s.dbgap_accession AS dbgap_accession
+  UNION
+  MATCH (t:treatment_other)-[:of_treatment_other]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+  WHERE s.dbgap_accession = 'phs000471' AND 'Unknown' IN coalesce(p.race, [])
+  RETURN p.participant_id AS participant_id,
+         t.guid AS treatment_id,
+         CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
+         CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
+         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
+         reduce(text = '', item IN coalesce(t.other_treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_agent,
+         s.dbgap_accession AS dbgap_accession
+}
+RETURN participant_id AS `Participant ID`,
+       treatment_id AS `Treatment ID`,
+       age_start AS `Age at Treatment Start`,
+       age_end AS `Age at Treatment End`,
+       treatment_type AS `Treatment Type`,
+       treatment_agent AS `Treatment Agent`,
+       dbgap_accession AS `dbGaP Accession`
+ORDER BY treatment_id
 LIMIT 100;</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
     </row>
     <row r="7" ht="409.6" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SurvivalTab</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT
-    prt.participant_id AS "Participant Id",
-    srv.survival_id AS "Survival Id",
-    srv.last_known_survival_status AS "Last Known Survival Status",
-    CASE 
-    WHEN srv.age_at_last_known_survival_status = -999 THEN 'Not Reported'
-    WHEN srv.age_at_last_known_survival_status &gt;= 1000 THEN 
-        substr(srv.age_at_last_known_survival_status, 1, length(srv.age_at_last_known_survival_status) - 3) || ',' || substr(srv.age_at_last_known_survival_status, -3)
-    ELSE 
-        srv.age_at_last_known_survival_status 
-END AS "Age at Last Known Survival Status",
-    std.dbgap_accession AS "dbGaP Accession"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1   -- participants not directly linked to studies
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE
-    std.dbgap_accession = 'phs000466' AND prt.sex_at_birth = 'Male' AND srv.survival_id IS NOT NULL
-ORDER BY 
-   srv.survival_id ASC
+          <t>TreatmentRespTab</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MATCH (tr:treatment_response)-[:of_treatment_response]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000471'
+  AND 'Unknown' IN coalesce(p.race, [])
+RETURN p.participant_id AS `Participant ID`,
+       tr.treatment_response_id AS `Treatment Response ID`,
+       reduce(text = '', item IN coalesce(tr.response, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS `Response`,
+       CASE
+         WHEN tr.age_at_response IS NULL OR tr.age_at_response = -999 THEN 'Not Reported'
+         ELSE toString(tr.age_at_response)
+       END AS `Age at Response`,
+       s.dbgap_accession AS `dbGaP Accession`
+ORDER BY p.participant_id
 LIMIT 100;</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GeneticAnalysisTab</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT
-    prt.participant_id AS "Participant Id",
-    ga.genetic_analysis_id AS "Genetic Analysis ID",
-    ga.gene_symbol AS "Gene Symbol",
-    ga.status AS "Status",
-    ga.reported_significance AS "Reported Significance",
-    ga.reported_significance_system AS "Reported Significance System",
-    ga.hgvs_genome AS "HGVS Genome",
-    ga.alteration AS "Alteration",
-    std.dbgap_accession AS "dbGaP Accession"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE 
-     std.dbgap_accession = 'phs000466' AND prt.sex_at_birth = 'Male' AND dgn.diagnosis_id IS NOT NULL
-ORDER BY 
-    ga.genetic_analysis_id ASC
+          <t>SurvivalTab</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MATCH (sv:survival)-[:of_survival]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000471'
+  AND 'Unknown' IN coalesce(p.race, [])
+RETURN p.participant_id AS `Participant ID`,
+       sv.survival_id AS `Survival ID`,
+       sv.last_known_survival_status AS `Last Known Survival Status`,
+       CASE
+         WHEN sv.age_at_last_known_survival_status IS NULL OR sv.age_at_last_known_survival_status = -999 THEN 'Not Reported'
+         ELSE toString(sv.age_at_last_known_survival_status)
+       END AS `Age at Last Known Survival Status`,
+       s.dbgap_accession AS `dbGaP Accession`
+ORDER BY p.participant_id, sv.survival_id
 LIMIT 100;</t>
         </is>
       </c>
-      <c r="C8" s="1" t="n"/>
     </row>
     <row r="9">
-      <c r="C9" s="1" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SamplesTab</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MATCH (sm:sample)-[:of_sample]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000471'
+  AND 'Unknown' IN coalesce(p.race, [])
+RETURN p.participant_id AS `Participant ID`,
+       sm.sample_id AS `Sample ID`,
+       s.study_id AS `Study ID`,
+       sm.tumor_spatial_extent AS `Tumor Spatial Extent`,
+       reduce(text = '', site IN coalesce(sm.anatomic_site, []) | CASE WHEN text = '' THEN site ELSE text + ';' + site END) AS `Anatomic Site`,
+       CASE
+         WHEN sm.participant_age_at_collection IS NULL OR sm.participant_age_at_collection = -999 THEN 'Not Reported'
+         ELSE toString(sm.participant_age_at_collection)
+       END AS `Participant Age at Collection (days)`,
+       sm.sample_tumor_status AS `Sample Tumor Status`
+ORDER BY sm.sample_id
+LIMIT 100;
+</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>